<commit_message>
feat(clearance): align public templates with MSDS fill style (layout + placeholders)
</commit_message>
<xml_diff>
--- a/references/clearance/CI-public.xlsx
+++ b/references/clearance/CI-public.xlsx
@@ -17,7 +17,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -25,16 +25,40 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E2F3"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -42,12 +66,132 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,318 +557,407 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:F33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+  </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>{{COMPANY_NAME_EN}}</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="2" t="inlineStr">
         <is>
           <t>{{COMPANY_ADDR_EN}}</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>{{COMPANY_TEL_EN}}</t>
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>TRANSPORT AND ROUTE：</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>{{ROUTE}}</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>CONTAINER NO.: {{CONTAINER_NO}}</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>SEAL NO.: {{SEAL_NO}}</t>
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>COMMERCIAL INVOICE</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="5" t="inlineStr">
         <is>
           <t>TO:</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="B11" s="5" t="inlineStr">
         <is>
           <t>{{CONSIGNEE_NAME}}</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>INVOICE NO.:</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>{{INVOICE_NO}}</t>
         </is>
       </c>
+      <c r="F11" s="6" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr"/>
-      <c r="B12" t="inlineStr">
+      <c r="A12" s="5" t="n"/>
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>{{CONSIGNEE_ADDR}} {{CONSIGNEE_TAX}}</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr">
+      <c r="C12" s="7" t="n"/>
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>DATE:</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr">
+      <c r="E12" s="5" t="inlineStr">
         <is>
           <t>{{INVOICE_DATE}}</t>
         </is>
       </c>
+      <c r="F12" s="6" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr">
+      <c r="A13" s="5" t="n"/>
+      <c r="B13" s="8" t="n"/>
+      <c r="C13" s="9" t="n"/>
+      <c r="D13" s="5" t="inlineStr">
         <is>
           <t>PI NO.:</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr">
+      <c r="E13" s="5" t="inlineStr">
         <is>
           <t>{{PI_NO}}</t>
         </is>
       </c>
+      <c r="F13" s="6" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="inlineStr">
+      <c r="A14" s="5" t="n"/>
+      <c r="B14" s="10" t="n"/>
+      <c r="C14" s="11" t="n"/>
+      <c r="D14" s="5" t="inlineStr">
         <is>
           <t>PRICE TERM:</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr">
+      <c r="E14" s="5" t="inlineStr">
         <is>
           <t>{{PRICE_TERM}}</t>
         </is>
       </c>
-    </row>
-    <row r="15"/>
-    <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="F14" s="6" t="n"/>
+    </row>
+    <row r="16" ht="28" customHeight="1">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>ITEM</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>DESCRIPTION</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr">
+      <c r="C16" s="12" t="inlineStr">
         <is>
           <t>QUANTITY</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr">
+      <c r="D16" s="12" t="inlineStr">
         <is>
           <t>CIF PRICE</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr">
+      <c r="E16" s="12" t="inlineStr">
         <is>
           <t>AMOUNT</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr"/>
-      <c r="B17" t="inlineStr"/>
-      <c r="C17" t="inlineStr">
+      <c r="A17" s="13" t="n"/>
+      <c r="B17" s="13" t="n"/>
+      <c r="C17" s="13" t="inlineStr">
         <is>
           <t>(KGS)</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>(USD)</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>(USD)</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="5" t="inlineStr">
         <is>
           <t>1</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>{{ITEM_DESC}}</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>{{ITEM_QTY}}</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>{{ITEM_PRICE}}</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr">
+      <c r="E18" s="5" t="inlineStr">
         <is>
           <t>{{ITEM_AMOUNT}}</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr"/>
-      <c r="B19" t="inlineStr">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="inlineStr">
         <is>
           <t>HS CODE: {{HS_CODES}}</t>
         </is>
       </c>
+      <c r="C19" s="2" t="n"/>
+      <c r="D19" s="2" t="n"/>
+      <c r="E19" s="2" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr"/>
-      <c r="B20" t="inlineStr">
+      <c r="A20" s="2" t="n"/>
+      <c r="B20" s="2" t="inlineStr">
         <is>
           <t>{{PO_LINE}}</t>
         </is>
       </c>
+      <c r="C20" s="2" t="n"/>
+      <c r="D20" s="2" t="n"/>
+      <c r="E20" s="2" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr"/>
-      <c r="B21" t="inlineStr">
+      <c r="A21" s="2" t="n"/>
+      <c r="B21" s="2" t="inlineStr">
         <is>
           <t>{{TOTALS_LINE}}</t>
         </is>
       </c>
+      <c r="C21" s="2" t="n"/>
+      <c r="D21" s="2" t="n"/>
+      <c r="E21" s="2" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE1}}</t>
         </is>
       </c>
+      <c r="B22" s="2" t="n"/>
+      <c r="C22" s="2" t="n"/>
+      <c r="D22" s="2" t="n"/>
+      <c r="E22" s="2" t="n"/>
+      <c r="F22" s="2" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE2}}</t>
         </is>
       </c>
+      <c r="B23" s="2" t="n"/>
+      <c r="C23" s="2" t="n"/>
+      <c r="D23" s="2" t="n"/>
+      <c r="E23" s="2" t="n"/>
+      <c r="F23" s="2" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE3}}</t>
         </is>
       </c>
+      <c r="B24" s="2" t="n"/>
+      <c r="C24" s="2" t="n"/>
+      <c r="D24" s="2" t="n"/>
+      <c r="E24" s="2" t="n"/>
+      <c r="F24" s="2" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" t="inlineStr">
+      <c r="A25" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE4}}</t>
         </is>
       </c>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+      <c r="F25" s="2" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE5}}</t>
         </is>
       </c>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
+      <c r="F26" s="2" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" t="inlineStr">
+      <c r="A27" s="2" t="inlineStr">
         <is>
           <t>{{BANK_LINE6}}</t>
         </is>
       </c>
+      <c r="B27" s="2" t="n"/>
+      <c r="C27" s="2" t="n"/>
+      <c r="D27" s="2" t="n"/>
+      <c r="E27" s="2" t="n"/>
+      <c r="F27" s="2" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" t="inlineStr">
+      <c r="A28" s="2" t="inlineStr">
         <is>
           <t>PAYMENT TERMS: {{PAYMENT_TERMS}}</t>
         </is>
       </c>
-    </row>
-    <row r="29"/>
+      <c r="B28" s="2" t="n"/>
+      <c r="C28" s="2" t="n"/>
+      <c r="D28" s="2" t="n"/>
+      <c r="E28" s="2" t="n"/>
+      <c r="F28" s="2" t="n"/>
+    </row>
     <row r="30">
-      <c r="A30" t="inlineStr">
+      <c r="A30" s="14" t="inlineStr">
         <is>
           <t>TOTAL:</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B30" s="14" t="inlineStr">
         <is>
           <t>{{TOTAL_QTY}}</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr">
+      <c r="C30" s="14" t="n"/>
+      <c r="D30" s="14" t="n"/>
+      <c r="E30" s="14" t="inlineStr">
         <is>
           <t>{{TOTAL_AMOUNT}}</t>
         </is>
       </c>
+      <c r="F30" s="6" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" t="inlineStr">
+      <c r="A31" s="2" t="inlineStr">
         <is>
           <t>{{AMOUNT_WORDS}}</t>
         </is>
       </c>
-    </row>
-    <row r="32"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
+      <c r="F31" s="2" t="n"/>
+    </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
+      <c r="E33" s="15" t="inlineStr">
         <is>
           <t>{{COMPANY_NAME_EN}}</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <mergeCells count="26">
+    <mergeCell ref="E12:F12"/>
+    <mergeCell ref="A27:F27"/>
+    <mergeCell ref="E14:F14"/>
+    <mergeCell ref="B20:E20"/>
+    <mergeCell ref="A3:F3"/>
+    <mergeCell ref="A26:F26"/>
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="B12:C14"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="A5:F5"/>
+    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A23:F23"/>
+    <mergeCell ref="A22:F22"/>
+    <mergeCell ref="E13:F13"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="A28:F28"/>
+    <mergeCell ref="E30:F30"/>
+    <mergeCell ref="E11:F11"/>
+    <mergeCell ref="B21:E21"/>
+    <mergeCell ref="A31:F31"/>
+    <mergeCell ref="A24:F24"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="A6:F6"/>
+    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="A25:F25"/>
+  </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>